<commit_message>
Los Excel de objetivos se llaman "2026-10 objetivos.xlsx"
La lista de costos del mismo mes se llama 2026-10.xlsx a secas, y los
dos archivos andan juntos por el escritorio y las descargas antes de
subirse: el nombre era lo unico que los distinguia, y no los distinguia.

Se acepta tambien con guion o guion bajo y el mes pelado, para que
renombrar no deje un archivo afuera. Dos archivos del mismo mes frenan
la carga: pasa al renombrar y olvidarse el viejo, y elegir uno seria
adivinar. "2026-10-18.xlsx", una lista de costos de media de mes subida
a la carpeta equivocada, se ignora.

2026-08 y 2026-09 se renombran; los datos no cambian.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDd85Xxe1Soek5dMXtHEjK
</commit_message>
<xml_diff>
--- a/objetivos_mensuales/PLANTILLA.xlsx
+++ b/objetivos_mensuales/PLANTILLA.xlsx
@@ -3028,7 +3028,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Una fila por objetivo. El archivo se llama como el mes comercial (2026-10.xlsx) y va en la carpeta objetivos_mensuales del repo tablero_quo.</t>
+          <t>Una fila por objetivo. El archivo se llama con el mes comercial: «2026-10 objetivos.xlsx» y va en la carpeta objetivos_mensuales del repo tablero_quo.</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Copiar el archivo del mes anterior, renombrarlo (2026-11.xlsx), cambiar MES_COMERCIAL en todas las filas y ajustar los numeros.</t>
+          <t>Copiar el archivo del mes anterior, renombrarlo («2026-11 objetivos.xlsx»), cambiar MES_COMERCIAL en todas las filas y ajustar los numeros.</t>
         </is>
       </c>
     </row>

</xml_diff>